<commit_message>
feat(integrations): sync engine, synthetic sandbox, Sync now (PI2b part 1) [R-5.1.2, R-7.3.3, R-7.5.1] (#98)
PI2b part 1: withTenantAsSystem, in-process synthetic FHIR sandbox, sync run
(paging, retries, page commits, field-encrypted member IDs, SSN/MBI refusal,
practice-local dates), Sync now, and migration 0043 (service principal,
owner-approved under R-15.9 on 2026-09-29). Real EHR connections fail closed
(population_scope_unenforced) until PI4.

AI-Assisted: true
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY7r13quPdzAWKCKUiLCt2
</commit_message>
<xml_diff>
--- a/docs/data-sources.xlsx
+++ b/docs/data-sources.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="25000" windowHeight="10000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Data sources" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,7 +12,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data sources'!$A$1:$P$13</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -30,12 +29,12 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -45,7 +44,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -56,6 +55,9 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F3A5F"/>
       </patternFill>
+    </fill>
+    <fill>
+      <patternFill/>
     </fill>
   </fills>
   <borders count="1">
@@ -68,25 +70,25 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -448,7 +450,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -458,8 +460,7 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="9" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="32" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
@@ -790,7 +791,7 @@
           <t>Owner: vendor choice</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1114,7 +1115,7 @@
           <t>Practice admin</t>
         </is>
       </c>
-      <c r="P8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1192,7 +1193,7 @@
           <t>Owner: vendor choice</t>
         </is>
       </c>
-      <c r="P9" s="2" t="inlineStr"/>
+      <c r="P9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1270,7 +1271,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1348,7 +1349,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1426,7 +1427,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1451,7 +1452,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>HL7 FHIR R4 (4.0.1), US Core 6.1.0 Patient + Coverage (+ Organization for payor names); SMART App Launch v2 Backend Services (private_key_jwt); later FHIR Bulk Data 2.0 Group/$export</t>
+          <t>HL7 FHIR R4 (4.0.1), US Core 6.1.0 Patient + Coverage (the payor name is the Coverage payor's own `display`; no Organization resource is fetched yet, its read scope is requested for a later lookup); SMART App Launch v2 Backend Services (private_key_jwt); later FHIR Bulk Data 2.0 Group/$export</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1486,7 +1487,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Built-in in-process synthetic FHIR sandbox (SYN- identifiers); vendor sandboxes pending OA-049</t>
+          <t>Built-in in-process synthetic FHIR sandbox (`SandboxTransport`, 125 Synthea-style patients, SYN- MRNs and member IDs, verifies the SMART client assertion); vendor sandboxes pending OA-049</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1496,17 +1497,17 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Designed (spec approved 2026-09-27; PI1-PI4 to build)</t>
+          <t>Sync engine and sandbox built (PI2b part 1: Sync now, in-request). The sync refuses every real connection (population_scope_unenforced) until PI4 applies the population scope; scheduled jobs, Coverage-only search, Bulk Data (PI3, PI4) not built</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Owner: OA-045, OA-046, OA-049, OA-050, OA-051, OA-052</t>
+          <t>Owner: OA-045, OA-046, OA-049, OA-050, OA-051, OA-052, OA-077, OA-078, OA-079, OA-080, OA-081, OA-082</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>ADR 0010; threat model docs/threat-models/patient-integrations.md. Signing key in platform key store, never in the database.</t>
+          <t>ADR 0010; threat model docs/threat-models/patient-integrations.md. Signing key in platform key store, never in the database. The sync writes as the integration service principal (migration 0043, OA-076). Coverage by POST search where supported.</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1595,10 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:P13"/>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="N10:N200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Needed,Stubbed (manual upload),Partial,Partial (CSV import),Connected,Connected (upload),Pending counsel verification,Retired"</formula1>
+    </dataValidation>
     <dataValidation sqref="N2:N200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Needed,Stubbed (manual upload),Partial,Partial (CSV import),Connected,Connected (upload),Pending counsel verification,Retired"</formula1>
     </dataValidation>
@@ -1610,7 +1614,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>

</xml_diff>